<commit_message>
Update soccer trades 2026-08-07 06:03:10 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Eredivisie/trades.xlsx
+++ b/data/sxbet/ligas/Eredivisie/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V3"/>
+  <dimension ref="A1:V4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,28 +531,28 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xbe3757de0d107fa27fec050f220d2720a303c2274c5053b041e64a8587c5429d</t>
+          <t>0x763d8974248de39c38179dce6fdf8aabf07c45a9532c44fd941f4ecaa4053020</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>42.19</t>
+          <t>14.19</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.6338</t>
+          <t>1.5675</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
+          <t>Asian Handicap (-2.5)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
@@ -563,27 +563,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Cambuur vs Excelsior Rotterdam FC</t>
+          <t>PSV Eindhoven vs Fortuna Sittard</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Cambuur</t>
+          <t>PSV Eindhoven</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Excelsior Rotterdam FC</t>
+          <t>Fortuna Sittard</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x5f73abff6c3a4dcbae7549384a24a6e32ed4fba83d1f8b6c07a54368215ec4b8</t>
+          <t>0x793b0538f962d70a57b2c5c4acd58d7dd39a82bb4331ea1b3fa94033d70c07e7</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19403942</t>
+          <t>L19403946</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -608,17 +608,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786044588</t>
+          <t>1786076493</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1786125600</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>66.571992</t>
+          <t>25.004405</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,110 +635,214 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>0xbe3757de0d107fa27fec050f220d2720a303c2274c5053b041e64a8587c5429d</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>42.19</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1.6338</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Eredivisie</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Cambuur vs Excelsior Rotterdam FC</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Cambuur</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Excelsior Rotterdam FC</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>0x5f73abff6c3a4dcbae7549384a24a6e32ed4fba83d1f8b6c07a54368215ec4b8</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>L19403942</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>1786044588</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>1786125600</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>66.571992</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>0x4ca810464ed1f6cc74ea5318f5d93dec93f4b441fa85a47c53e1f17f3dc3f2ff</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>35.25</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>1.195</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Tie</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>Eredivisie</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>NEC Nijmegen vs SC Telstar</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>NEC Nijmegen</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>SC Telstar</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>0x32e22d2bad4d17213f93e2773019169fc54af66f0156ef2678851d836d908f54</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>L19403940</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>1786038454</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>1786199400</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t>180.769231</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr">
+      <c r="V4" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-07 07:02:35 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Eredivisie/trades.xlsx
+++ b/data/sxbet/ligas/Eredivisie/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V4"/>
+  <dimension ref="A1:V5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,31 +531,39 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x763d8974248de39c38179dce6fdf8aabf07c45a9532c44fd941f4ecaa4053020</t>
+          <t>0x9f01fbafa94a70a9cf6ab60945073f6a9cfd9c030489c2f7ad0e408d82e12640</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
+          <t>0xcF597434D48cDA55032b9d4931a0FFAeeEe7fb0D</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>14.19</t>
+          <t>20.39624</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.5675</t>
+          <t>1.375</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Asian Handicap (-2.5)</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Excelsior Rotterdam FC</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>Eredivisie</t>
@@ -563,27 +571,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>PSV Eindhoven vs Fortuna Sittard</t>
+          <t>Cambuur vs Excelsior Rotterdam FC</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>PSV Eindhoven</t>
+          <t>Cambuur</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Fortuna Sittard</t>
+          <t>Excelsior Rotterdam FC</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x793b0538f962d70a57b2c5c4acd58d7dd39a82bb4331ea1b3fa94033d70c07e7</t>
+          <t>0xaa0c126d35fe767a756910f2acec4006318f8fe1dab75625727393f8adb31b74</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19403946</t>
+          <t>L19403942</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -608,17 +616,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786076493</t>
+          <t>1786082661</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786125600</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>25.004405</t>
+          <t>54.389973</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,28 +643,28 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0xbe3757de0d107fa27fec050f220d2720a303c2274c5053b041e64a8587c5429d</t>
+          <t>0x763d8974248de39c38179dce6fdf8aabf07c45a9532c44fd941f4ecaa4053020</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>42.19</t>
+          <t>14.19</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.6338</t>
+          <t>1.5675</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
+          <t>Asian Handicap (-2.5)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
@@ -667,27 +675,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Cambuur vs Excelsior Rotterdam FC</t>
+          <t>PSV Eindhoven vs Fortuna Sittard</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Cambuur</t>
+          <t>PSV Eindhoven</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Excelsior Rotterdam FC</t>
+          <t>Fortuna Sittard</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x5f73abff6c3a4dcbae7549384a24a6e32ed4fba83d1f8b6c07a54368215ec4b8</t>
+          <t>0x793b0538f962d70a57b2c5c4acd58d7dd39a82bb4331ea1b3fa94033d70c07e7</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19403942</t>
+          <t>L19403946</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -712,17 +720,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786044588</t>
+          <t>1786076493</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1786125600</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>66.571992</t>
+          <t>25.004405</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -739,110 +747,214 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>0xbe3757de0d107fa27fec050f220d2720a303c2274c5053b041e64a8587c5429d</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>42.19</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>1.6338</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Eredivisie</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Cambuur vs Excelsior Rotterdam FC</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Cambuur</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Excelsior Rotterdam FC</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>0x5f73abff6c3a4dcbae7549384a24a6e32ed4fba83d1f8b6c07a54368215ec4b8</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>L19403942</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>1786044588</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>1786125600</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>66.571992</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t>0x4ca810464ed1f6cc74ea5318f5d93dec93f4b441fa85a47c53e1f17f3dc3f2ff</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>35.25</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>1.195</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Tie</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>Eredivisie</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>NEC Nijmegen vs SC Telstar</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>NEC Nijmegen</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>SC Telstar</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>0x32e22d2bad4d17213f93e2773019169fc54af66f0156ef2678851d836d908f54</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>L19403940</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="Q5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="R5" t="inlineStr">
         <is>
           <t>1786038454</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="S5" t="inlineStr">
         <is>
           <t>1786199400</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="T5" t="inlineStr">
         <is>
           <t>180.769231</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="U5" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr">
+      <c r="V5" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-07 08:03:35 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Eredivisie/trades.xlsx
+++ b/data/sxbet/ligas/Eredivisie/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V5"/>
+  <dimension ref="A1:V6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,12 +531,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x9f01fbafa94a70a9cf6ab60945073f6a9cfd9c030489c2f7ad0e408d82e12640</t>
+          <t>0xd6c7c9abba838597a4e77b3e2783253562734141d39ee275990cdeca84ed5917</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0xcF597434D48cDA55032b9d4931a0FFAeeEe7fb0D</t>
+          <t>0x8Aba6E6af9321Edf3b1b3b1CA92adEdb93D247C6</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -546,47 +546,47 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>20.39624</t>
+          <t>173</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.375</t>
+          <t>1.3438</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (3.5)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
+          <t>Over 3.5</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Eredivisie</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Cambuur vs Excelsior Rotterdam FC</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Cambuur</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
           <t>Excelsior Rotterdam FC</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Eredivisie</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Cambuur vs Excelsior Rotterdam FC</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Cambuur</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Excelsior Rotterdam FC</t>
-        </is>
-      </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0xaa0c126d35fe767a756910f2acec4006318f8fe1dab75625727393f8adb31b74</t>
+          <t>0x5f73abff6c3a4dcbae7549384a24a6e32ed4fba83d1f8b6c07a54368215ec4b8</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -616,7 +616,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786082661</t>
+          <t>1786086947</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -626,7 +626,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>54.389973</t>
+          <t>503.272727</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,31 +643,39 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x763d8974248de39c38179dce6fdf8aabf07c45a9532c44fd941f4ecaa4053020</t>
+          <t>0x9f01fbafa94a70a9cf6ab60945073f6a9cfd9c030489c2f7ad0e408d82e12640</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
+          <t>0xcF597434D48cDA55032b9d4931a0FFAeeEe7fb0D</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>14.19</t>
+          <t>20.39624</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.5675</t>
+          <t>1.375</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Asian Handicap (-2.5)</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Excelsior Rotterdam FC</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>Eredivisie</t>
@@ -675,27 +683,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>PSV Eindhoven vs Fortuna Sittard</t>
+          <t>Cambuur vs Excelsior Rotterdam FC</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>PSV Eindhoven</t>
+          <t>Cambuur</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Fortuna Sittard</t>
+          <t>Excelsior Rotterdam FC</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x793b0538f962d70a57b2c5c4acd58d7dd39a82bb4331ea1b3fa94033d70c07e7</t>
+          <t>0xaa0c126d35fe767a756910f2acec4006318f8fe1dab75625727393f8adb31b74</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19403946</t>
+          <t>L19403942</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -720,17 +728,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786076493</t>
+          <t>1786082661</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786125600</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>25.004405</t>
+          <t>54.389973</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -747,28 +755,28 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0xbe3757de0d107fa27fec050f220d2720a303c2274c5053b041e64a8587c5429d</t>
+          <t>0x763d8974248de39c38179dce6fdf8aabf07c45a9532c44fd941f4ecaa4053020</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>42.19</t>
+          <t>14.19</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.6338</t>
+          <t>1.5675</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
+          <t>Asian Handicap (-2.5)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
@@ -779,27 +787,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Cambuur vs Excelsior Rotterdam FC</t>
+          <t>PSV Eindhoven vs Fortuna Sittard</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Cambuur</t>
+          <t>PSV Eindhoven</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Excelsior Rotterdam FC</t>
+          <t>Fortuna Sittard</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x5f73abff6c3a4dcbae7549384a24a6e32ed4fba83d1f8b6c07a54368215ec4b8</t>
+          <t>0x793b0538f962d70a57b2c5c4acd58d7dd39a82bb4331ea1b3fa94033d70c07e7</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19403942</t>
+          <t>L19403946</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -824,17 +832,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786044588</t>
+          <t>1786076493</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1786125600</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>66.571992</t>
+          <t>25.004405</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -851,110 +859,214 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>0xbe3757de0d107fa27fec050f220d2720a303c2274c5053b041e64a8587c5429d</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>42.19</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1.6338</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Eredivisie</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Cambuur vs Excelsior Rotterdam FC</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Cambuur</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Excelsior Rotterdam FC</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>0x5f73abff6c3a4dcbae7549384a24a6e32ed4fba83d1f8b6c07a54368215ec4b8</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>L19403942</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>1786044588</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>1786125600</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>66.571992</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t>0x4ca810464ed1f6cc74ea5318f5d93dec93f4b441fa85a47c53e1f17f3dc3f2ff</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>35.25</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>1.195</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>Tie</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>Eredivisie</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>NEC Nijmegen vs SC Telstar</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>NEC Nijmegen</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>SC Telstar</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>0x32e22d2bad4d17213f93e2773019169fc54af66f0156ef2678851d836d908f54</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>L19403940</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="P6" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr">
+      <c r="Q6" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="R6" t="inlineStr">
         <is>
           <t>1786038454</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
+      <c r="S6" t="inlineStr">
         <is>
           <t>1786199400</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr">
+      <c r="T6" t="inlineStr">
         <is>
           <t>180.769231</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
+      <c r="U6" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr">
+      <c r="V6" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-07 11:03:02 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Eredivisie/trades.xlsx
+++ b/data/sxbet/ligas/Eredivisie/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V6"/>
+  <dimension ref="A1:V8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,12 +531,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xd6c7c9abba838597a4e77b3e2783253562734141d39ee275990cdeca84ed5917</t>
+          <t>0xe3ab30d6b781a9a79b98b5a3c156060adf02a4cb6dd79257d045954564c464f4</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x8Aba6E6af9321Edf3b1b3b1CA92adEdb93D247C6</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -546,22 +546,22 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>173</t>
+          <t>54.37</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.3438</t>
+          <t>1.3588</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Over 3.5</t>
+          <t>Excelsior Rotterdam FC</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -586,7 +586,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x5f73abff6c3a4dcbae7549384a24a6e32ed4fba83d1f8b6c07a54368215ec4b8</t>
+          <t>0xaa0c126d35fe767a756910f2acec4006318f8fe1dab75625727393f8adb31b74</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -616,7 +616,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786086947</t>
+          <t>1786096483</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -626,7 +626,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>503.272727</t>
+          <t>151.554007</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,12 +643,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x9f01fbafa94a70a9cf6ab60945073f6a9cfd9c030489c2f7ad0e408d82e12640</t>
+          <t>0xfcb42550a86c19b2c5cb5270b8fbf7ab1826b37014cd165720a9eba42002beba</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0xcF597434D48cDA55032b9d4931a0FFAeeEe7fb0D</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -658,12 +658,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>20.39624</t>
+          <t>5.63</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.375</t>
+          <t>1.3588</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -728,7 +728,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786082661</t>
+          <t>1786095316</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -738,7 +738,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>54.389973</t>
+          <t>15.69338</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -755,31 +755,39 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x763d8974248de39c38179dce6fdf8aabf07c45a9532c44fd941f4ecaa4053020</t>
+          <t>0xd6c7c9abba838597a4e77b3e2783253562734141d39ee275990cdeca84ed5917</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
+          <t>0x8Aba6E6af9321Edf3b1b3b1CA92adEdb93D247C6</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>14.19</t>
+          <t>173</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.5675</t>
+          <t>1.3438</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Asian Handicap (-2.5)</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Over 3.5</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>Eredivisie</t>
@@ -787,27 +795,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>PSV Eindhoven vs Fortuna Sittard</t>
+          <t>Cambuur vs Excelsior Rotterdam FC</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>PSV Eindhoven</t>
+          <t>Cambuur</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Fortuna Sittard</t>
+          <t>Excelsior Rotterdam FC</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x793b0538f962d70a57b2c5c4acd58d7dd39a82bb4331ea1b3fa94033d70c07e7</t>
+          <t>0x5f73abff6c3a4dcbae7549384a24a6e32ed4fba83d1f8b6c07a54368215ec4b8</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19403946</t>
+          <t>L19403942</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -832,17 +840,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786076493</t>
+          <t>1786086947</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786125600</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>25.004405</t>
+          <t>503.272727</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -859,31 +867,39 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0xbe3757de0d107fa27fec050f220d2720a303c2274c5053b041e64a8587c5429d</t>
+          <t>0x9f01fbafa94a70a9cf6ab60945073f6a9cfd9c030489c2f7ad0e408d82e12640</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
+          <t>0xcF597434D48cDA55032b9d4931a0FFAeeEe7fb0D</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>42.19</t>
+          <t>20.39624</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.6338</t>
+          <t>1.375</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Excelsior Rotterdam FC</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>Eredivisie</t>
@@ -906,7 +922,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0x5f73abff6c3a4dcbae7549384a24a6e32ed4fba83d1f8b6c07a54368215ec4b8</t>
+          <t>0xaa0c126d35fe767a756910f2acec4006318f8fe1dab75625727393f8adb31b74</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -936,7 +952,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786044588</t>
+          <t>1786082661</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -946,7 +962,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>66.571992</t>
+          <t>54.389973</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -963,110 +979,318 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>0x763d8974248de39c38179dce6fdf8aabf07c45a9532c44fd941f4ecaa4053020</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>14.19</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>1.5675</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-2.5)</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Eredivisie</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>PSV Eindhoven vs Fortuna Sittard</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>PSV Eindhoven</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Fortuna Sittard</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>0x793b0538f962d70a57b2c5c4acd58d7dd39a82bb4331ea1b3fa94033d70c07e7</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>L19403946</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>1786076493</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>1786212000</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>25.004405</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>0xbe3757de0d107fa27fec050f220d2720a303c2274c5053b041e64a8587c5429d</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>42.19</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>1.6338</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Eredivisie</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Cambuur vs Excelsior Rotterdam FC</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Cambuur</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Excelsior Rotterdam FC</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>0x5f73abff6c3a4dcbae7549384a24a6e32ed4fba83d1f8b6c07a54368215ec4b8</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>L19403942</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>1786044588</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>1786125600</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>66.571992</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>0x4ca810464ed1f6cc74ea5318f5d93dec93f4b441fa85a47c53e1f17f3dc3f2ff</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>35.25</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>1.195</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>Tie</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>Eredivisie</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>NEC Nijmegen vs SC Telstar</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>NEC Nijmegen</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>SC Telstar</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>0x32e22d2bad4d17213f93e2773019169fc54af66f0156ef2678851d836d908f54</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>L19403940</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="P8" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr">
+      <c r="Q8" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr">
+      <c r="R8" t="inlineStr">
         <is>
           <t>1786038454</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr">
+      <c r="S8" t="inlineStr">
         <is>
           <t>1786199400</t>
         </is>
       </c>
-      <c r="T6" t="inlineStr">
+      <c r="T8" t="inlineStr">
         <is>
           <t>180.769231</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr">
+      <c r="U8" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V6" t="inlineStr">
+      <c r="V8" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-07 14:02:46 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Eredivisie/trades.xlsx
+++ b/data/sxbet/ligas/Eredivisie/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V8"/>
+  <dimension ref="A1:V15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,12 +531,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xe3ab30d6b781a9a79b98b5a3c156060adf02a4cb6dd79257d045954564c464f4</t>
+          <t>0x5814ac08c32ab173d1a31814cb3a6b884d7c9919e8f377ee4f05aeaa32cb47ee</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0xCf35f1782f282b1c6659882a3FAA48C637Ab693b</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -546,12 +546,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>54.37</t>
+          <t>9.99999</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.3588</t>
+          <t>1.5888</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -561,7 +561,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Excelsior Rotterdam FC</t>
+          <t>Go Ahead Eagles</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -571,27 +571,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Cambuur vs Excelsior Rotterdam FC</t>
+          <t>Go Ahead Eagles vs Willem II Tilburg</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Cambuur</t>
+          <t>Go Ahead Eagles</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Excelsior Rotterdam FC</t>
+          <t>Willem II Tilburg</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0xaa0c126d35fe767a756910f2acec4006318f8fe1dab75625727393f8adb31b74</t>
+          <t>0x8aa5f120fe51985c65586c394c669657f5118efb952dee047f9dabfcbeb011d3</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19403942</t>
+          <t>L19403947</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -616,17 +616,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786096483</t>
+          <t>1786105696</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1786125600</t>
+          <t>1786207500</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>151.554007</t>
+          <t>16.985121</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,12 +643,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0xfcb42550a86c19b2c5cb5270b8fbf7ab1826b37014cd165720a9eba42002beba</t>
+          <t>0xf98e5cfa7926a69ff6e557c416734c337a5cb9347da000cf0a1b8afd308312c1</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0xCf35f1782f282b1c6659882a3FAA48C637Ab693b</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -658,22 +658,22 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>5.63</t>
+          <t>4.49993</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.3588</t>
+          <t>1.9463</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (0.5)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Excelsior Rotterdam FC</t>
+          <t>Over 0.5</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -683,7 +683,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Cambuur vs Excelsior Rotterdam FC</t>
+          <t>Cambuur vs Excelsior Rotterdam</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -693,12 +693,12 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Excelsior Rotterdam FC</t>
+          <t>Excelsior Rotterdam</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0xaa0c126d35fe767a756910f2acec4006318f8fe1dab75625727393f8adb31b74</t>
+          <t>0x1decb278c23c8109eb9cf89c45fcff13cc3065960479465ded1dc8684e6e3f1f</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -728,7 +728,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786095316</t>
+          <t>1786104752</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -738,7 +738,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>15.69338</t>
+          <t>4.75554</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -755,12 +755,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0xd6c7c9abba838597a4e77b3e2783253562734141d39ee275990cdeca84ed5917</t>
+          <t>0x85052153f0e8ac58dbcbeb02f546bbc166e1c5e3e8753d3dee4219a55150e22d</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x8Aba6E6af9321Edf3b1b3b1CA92adEdb93D247C6</t>
+          <t>0xCf35f1782f282b1c6659882a3FAA48C637Ab693b</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -770,22 +770,22 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>173</t>
+          <t>5.99989</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.3438</t>
+          <t>1.945</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
+          <t>Under/Over (0.5)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Over 3.5</t>
+          <t>Over 0.5</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -795,7 +795,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Cambuur vs Excelsior Rotterdam FC</t>
+          <t>Cambuur vs Excelsior Rotterdam</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -805,12 +805,12 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Excelsior Rotterdam FC</t>
+          <t>Excelsior Rotterdam</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x5f73abff6c3a4dcbae7549384a24a6e32ed4fba83d1f8b6c07a54368215ec4b8</t>
+          <t>0x1decb278c23c8109eb9cf89c45fcff13cc3065960479465ded1dc8684e6e3f1f</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -840,7 +840,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786086947</t>
+          <t>1786104743</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -850,7 +850,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>503.272727</t>
+          <t>6.34909</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -867,39 +867,31 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x9f01fbafa94a70a9cf6ab60945073f6a9cfd9c030489c2f7ad0e408d82e12640</t>
+          <t>0xc99b1deff403bd60532b3766c532f84759f6d39b1bdbf56a0da46442c81b8dbe</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0xcF597434D48cDA55032b9d4931a0FFAeeEe7fb0D</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xbFA1723b261cB748697a7FFc3236E1c7C04bfC5e</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>20.39624</t>
+          <t>2.27</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.375</t>
+          <t>1.6125</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Excelsior Rotterdam FC</t>
-        </is>
-      </c>
+          <t>Under/Over (4.5)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>Eredivisie</t>
@@ -907,27 +899,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Cambuur vs Excelsior Rotterdam FC</t>
+          <t>PSV Eindhoven vs Fortuna Sittard</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Cambuur</t>
+          <t>PSV Eindhoven</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Excelsior Rotterdam FC</t>
+          <t>Fortuna Sittard</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0xaa0c126d35fe767a756910f2acec4006318f8fe1dab75625727393f8adb31b74</t>
+          <t>0xd10635672e9e5618b0fee4290a52fdad51735dc4dfbd7ede4bc2a4e63cc90c47</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19403942</t>
+          <t>L19403946</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -952,17 +944,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786082661</t>
+          <t>1786102413</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>1786125600</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>54.389973</t>
+          <t>3.706122</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -979,28 +971,28 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x763d8974248de39c38179dce6fdf8aabf07c45a9532c44fd941f4ecaa4053020</t>
+          <t>0x557b8c1f5c5c8b5fb903d079ecd882cabc34a595be512242ec8c9f410dc89cc8</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+          <t>0xbFA1723b261cB748697a7FFc3236E1c7C04bfC5e</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>14.19</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.5675</t>
+          <t>1.2212</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Asian Handicap (-2.5)</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
@@ -1026,7 +1018,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0x793b0538f962d70a57b2c5c4acd58d7dd39a82bb4331ea1b3fa94033d70c07e7</t>
+          <t>0x655963edf32f16b3a45d6a00e88736f6309fec1474356ce20fc40bcb6fec13aa</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1056,7 +1048,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786076493</t>
+          <t>1786102412</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1066,7 +1058,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>25.004405</t>
+          <t>4.519774</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1083,23 +1075,23 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0xbe3757de0d107fa27fec050f220d2720a303c2274c5053b041e64a8587c5429d</t>
+          <t>0xd876072232054549cb6720da6ed0929158b37dc7f9e1ed70e03cf4bb6785214e</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0xbFA1723b261cB748697a7FFc3236E1c7C04bfC5e</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>42.19</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.6338</t>
+          <t>1.4138</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1115,27 +1107,27 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Cambuur vs Excelsior Rotterdam FC</t>
+          <t>PSV Eindhoven vs Fortuna Sittard</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Cambuur</t>
+          <t>PSV Eindhoven</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Excelsior Rotterdam FC</t>
+          <t>Fortuna Sittard</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x5f73abff6c3a4dcbae7549384a24a6e32ed4fba83d1f8b6c07a54368215ec4b8</t>
+          <t>0x8e63f170dc54d5f8c63f531a5dcccded818e9d9e5f10a9596397c42875b381c7</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>L19403942</t>
+          <t>L19403946</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1160,17 +1152,17 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786044588</t>
+          <t>1786102410</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>1786125600</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>66.571992</t>
+          <t>2.416918</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1187,110 +1179,870 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>0xfb67071ab7e9a27f540fd95f339b51a0fac006bd9950b6d733ec4be68c85bb16</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>0xbFA1723b261cB748697a7FFc3236E1c7C04bfC5e</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>1.195</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Eredivisie</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Go Ahead Eagles vs Willem II Tilburg</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Go Ahead Eagles</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Willem II Tilburg</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>0x850e00f49e80137284f56035827d7137ff8b0500f064e9bbebfb9172d34d807c</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>L19403947</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>1786102409</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>1786207500</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>5.128205</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>0xe3ab30d6b781a9a79b98b5a3c156060adf02a4cb6dd79257d045954564c464f4</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>54.37</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>1.3588</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Excelsior Rotterdam FC</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Eredivisie</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Cambuur vs Excelsior Rotterdam FC</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Cambuur</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Excelsior Rotterdam FC</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>0xaa0c126d35fe767a756910f2acec4006318f8fe1dab75625727393f8adb31b74</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>L19403942</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>1786096483</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>1786125600</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>151.554007</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>0xfcb42550a86c19b2c5cb5270b8fbf7ab1826b37014cd165720a9eba42002beba</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>5.63</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>1.3588</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Excelsior Rotterdam FC</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Eredivisie</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Cambuur vs Excelsior Rotterdam FC</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Cambuur</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Excelsior Rotterdam FC</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>0xaa0c126d35fe767a756910f2acec4006318f8fe1dab75625727393f8adb31b74</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>L19403942</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>1786095316</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>1786125600</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>15.69338</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>0xd6c7c9abba838597a4e77b3e2783253562734141d39ee275990cdeca84ed5917</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>0x8Aba6E6af9321Edf3b1b3b1CA92adEdb93D247C6</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>173</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>1.3438</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Over 3.5</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Eredivisie</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Cambuur vs Excelsior Rotterdam FC</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Cambuur</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Excelsior Rotterdam FC</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>0x5f73abff6c3a4dcbae7549384a24a6e32ed4fba83d1f8b6c07a54368215ec4b8</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>L19403942</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>1786086947</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>1786125600</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>503.272727</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>0x9f01fbafa94a70a9cf6ab60945073f6a9cfd9c030489c2f7ad0e408d82e12640</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>0xcF597434D48cDA55032b9d4931a0FFAeeEe7fb0D</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>20.39624</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>1.375</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Excelsior Rotterdam FC</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Eredivisie</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Cambuur vs Excelsior Rotterdam FC</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Cambuur</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Excelsior Rotterdam FC</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>0xaa0c126d35fe767a756910f2acec4006318f8fe1dab75625727393f8adb31b74</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>L19403942</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>1786082661</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>1786125600</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>54.389973</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>0x763d8974248de39c38179dce6fdf8aabf07c45a9532c44fd941f4ecaa4053020</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>14.19</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>1.5675</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-2.5)</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Eredivisie</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>PSV Eindhoven vs Fortuna Sittard</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>PSV Eindhoven</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Fortuna Sittard</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>0x793b0538f962d70a57b2c5c4acd58d7dd39a82bb4331ea1b3fa94033d70c07e7</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>L19403946</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>1786076493</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>1786212000</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>25.004405</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>0xbe3757de0d107fa27fec050f220d2720a303c2274c5053b041e64a8587c5429d</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>42.19</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>1.6338</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Eredivisie</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Cambuur vs Excelsior Rotterdam FC</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Cambuur</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Excelsior Rotterdam FC</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>0x5f73abff6c3a4dcbae7549384a24a6e32ed4fba83d1f8b6c07a54368215ec4b8</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>L19403942</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>1786044588</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>1786125600</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>66.571992</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>0x4ca810464ed1f6cc74ea5318f5d93dec93f4b441fa85a47c53e1f17f3dc3f2ff</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
         <is>
           <t>35.25</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>1.195</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>Tie</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>Eredivisie</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>NEC Nijmegen vs SC Telstar</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t>NEC Nijmegen</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>SC Telstar</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>0x32e22d2bad4d17213f93e2773019169fc54af66f0156ef2678851d836d908f54</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="M15" t="inlineStr">
         <is>
           <t>L19403940</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr">
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
         <is>
           <t>1786038454</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr">
+      <c r="S15" t="inlineStr">
         <is>
           <t>1786199400</t>
         </is>
       </c>
-      <c r="T8" t="inlineStr">
+      <c r="T15" t="inlineStr">
         <is>
           <t>180.769231</t>
         </is>
       </c>
-      <c r="U8" t="inlineStr">
+      <c r="U15" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V8" t="inlineStr">
+      <c r="V15" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-07 15:03:09 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Eredivisie/trades.xlsx
+++ b/data/sxbet/ligas/Eredivisie/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V15"/>
+  <dimension ref="A1:V16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,12 +531,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x5814ac08c32ab173d1a31814cb3a6b884d7c9919e8f377ee4f05aeaa32cb47ee</t>
+          <t>0x30e80e0f179988de24d2dd1521c00c47b8a96c2e0b127f5b72b5656e3f3c392a</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0xCf35f1782f282b1c6659882a3FAA48C637Ab693b</t>
+          <t>0xFe080e9732dfD21D183C50e533A0B4b16021512a</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -546,7 +546,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>9.99999</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -616,7 +616,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786105696</t>
+          <t>1786111515</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -626,7 +626,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>16.985121</t>
+          <t>1.698514</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,7 +643,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0xf98e5cfa7926a69ff6e557c416734c337a5cb9347da000cf0a1b8afd308312c1</t>
+          <t>0x5814ac08c32ab173d1a31814cb3a6b884d7c9919e8f377ee4f05aeaa32cb47ee</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -658,22 +658,22 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>4.49993</t>
+          <t>9.99999</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.9463</t>
+          <t>1.5888</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Under/Over (0.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Over 0.5</t>
+          <t>Go Ahead Eagles</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -683,27 +683,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Cambuur vs Excelsior Rotterdam</t>
+          <t>Go Ahead Eagles vs Willem II Tilburg</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Cambuur</t>
+          <t>Go Ahead Eagles</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Excelsior Rotterdam</t>
+          <t>Willem II Tilburg</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x1decb278c23c8109eb9cf89c45fcff13cc3065960479465ded1dc8684e6e3f1f</t>
+          <t>0x8aa5f120fe51985c65586c394c669657f5118efb952dee047f9dabfcbeb011d3</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19403942</t>
+          <t>L19403947</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -728,17 +728,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786104752</t>
+          <t>1786105696</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1786125600</t>
+          <t>1786207500</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>4.75554</t>
+          <t>16.985121</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -755,7 +755,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x85052153f0e8ac58dbcbeb02f546bbc166e1c5e3e8753d3dee4219a55150e22d</t>
+          <t>0xf98e5cfa7926a69ff6e557c416734c337a5cb9347da000cf0a1b8afd308312c1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -770,12 +770,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5.99989</t>
+          <t>4.49993</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.945</t>
+          <t>1.9463</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -840,7 +840,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786104743</t>
+          <t>1786104752</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -850,7 +850,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>6.34909</t>
+          <t>4.75554</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -867,31 +867,39 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0xc99b1deff403bd60532b3766c532f84759f6d39b1bdbf56a0da46442c81b8dbe</t>
+          <t>0x85052153f0e8ac58dbcbeb02f546bbc166e1c5e3e8753d3dee4219a55150e22d</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0xbFA1723b261cB748697a7FFc3236E1c7C04bfC5e</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
+          <t>0xCf35f1782f282b1c6659882a3FAA48C637Ab693b</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2.27</t>
+          <t>5.99989</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.6125</t>
+          <t>1.945</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Under/Over (4.5)</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
+          <t>Under/Over (0.5)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Over 0.5</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>Eredivisie</t>
@@ -899,27 +907,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>PSV Eindhoven vs Fortuna Sittard</t>
+          <t>Cambuur vs Excelsior Rotterdam</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>PSV Eindhoven</t>
+          <t>Cambuur</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Fortuna Sittard</t>
+          <t>Excelsior Rotterdam</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0xd10635672e9e5618b0fee4290a52fdad51735dc4dfbd7ede4bc2a4e63cc90c47</t>
+          <t>0x1decb278c23c8109eb9cf89c45fcff13cc3065960479465ded1dc8684e6e3f1f</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19403946</t>
+          <t>L19403942</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -944,17 +952,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786102413</t>
+          <t>1786104743</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786125600</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>3.706122</t>
+          <t>6.34909</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -971,7 +979,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x557b8c1f5c5c8b5fb903d079ecd882cabc34a595be512242ec8c9f410dc89cc8</t>
+          <t>0xc99b1deff403bd60532b3766c532f84759f6d39b1bdbf56a0da46442c81b8dbe</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -982,17 +990,17 @@
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2.27</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.2212</t>
+          <t>1.6125</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>Under/Over (4.5)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
@@ -1018,7 +1026,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0x655963edf32f16b3a45d6a00e88736f6309fec1474356ce20fc40bcb6fec13aa</t>
+          <t>0xd10635672e9e5618b0fee4290a52fdad51735dc4dfbd7ede4bc2a4e63cc90c47</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1048,7 +1056,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786102412</t>
+          <t>1786102413</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1058,7 +1066,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>4.519774</t>
+          <t>3.706122</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1075,7 +1083,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0xd876072232054549cb6720da6ed0929158b37dc7f9e1ed70e03cf4bb6785214e</t>
+          <t>0x557b8c1f5c5c8b5fb903d079ecd882cabc34a595be512242ec8c9f410dc89cc8</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1091,12 +1099,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.4138</t>
+          <t>1.2212</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
@@ -1122,7 +1130,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x8e63f170dc54d5f8c63f531a5dcccded818e9d9e5f10a9596397c42875b381c7</t>
+          <t>0x655963edf32f16b3a45d6a00e88736f6309fec1474356ce20fc40bcb6fec13aa</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1152,7 +1160,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786102410</t>
+          <t>1786102412</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1162,7 +1170,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>2.416918</t>
+          <t>4.519774</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1179,7 +1187,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0xfb67071ab7e9a27f540fd95f339b51a0fac006bd9950b6d733ec4be68c85bb16</t>
+          <t>0xd876072232054549cb6720da6ed0929158b37dc7f9e1ed70e03cf4bb6785214e</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1195,12 +1203,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.195</t>
+          <t>1.4138</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>Under/Over (3.5)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
@@ -1211,27 +1219,27 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Go Ahead Eagles vs Willem II Tilburg</t>
+          <t>PSV Eindhoven vs Fortuna Sittard</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Go Ahead Eagles</t>
+          <t>PSV Eindhoven</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Willem II Tilburg</t>
+          <t>Fortuna Sittard</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x850e00f49e80137284f56035827d7137ff8b0500f064e9bbebfb9172d34d807c</t>
+          <t>0x8e63f170dc54d5f8c63f531a5dcccded818e9d9e5f10a9596397c42875b381c7</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>L19403947</t>
+          <t>L19403946</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1256,17 +1264,17 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1786102409</t>
+          <t>1786102410</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>1786207500</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>5.128205</t>
+          <t>2.416918</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1283,39 +1291,31 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0xe3ab30d6b781a9a79b98b5a3c156060adf02a4cb6dd79257d045954564c464f4</t>
+          <t>0xfb67071ab7e9a27f540fd95f339b51a0fac006bd9950b6d733ec4be68c85bb16</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xbFA1723b261cB748697a7FFc3236E1c7C04bfC5e</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>54.37</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.3588</t>
+          <t>1.195</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Excelsior Rotterdam FC</t>
-        </is>
-      </c>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>Eredivisie</t>
@@ -1323,27 +1323,27 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Cambuur vs Excelsior Rotterdam FC</t>
+          <t>Go Ahead Eagles vs Willem II Tilburg</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Cambuur</t>
+          <t>Go Ahead Eagles</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Excelsior Rotterdam FC</t>
+          <t>Willem II Tilburg</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0xaa0c126d35fe767a756910f2acec4006318f8fe1dab75625727393f8adb31b74</t>
+          <t>0x850e00f49e80137284f56035827d7137ff8b0500f064e9bbebfb9172d34d807c</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>L19403942</t>
+          <t>L19403947</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1368,17 +1368,17 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1786096483</t>
+          <t>1786102409</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>1786125600</t>
+          <t>1786207500</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>151.554007</t>
+          <t>5.128205</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1395,7 +1395,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0xfcb42550a86c19b2c5cb5270b8fbf7ab1826b37014cd165720a9eba42002beba</t>
+          <t>0xe3ab30d6b781a9a79b98b5a3c156060adf02a4cb6dd79257d045954564c464f4</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1410,7 +1410,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>5.63</t>
+          <t>54.37</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1480,7 +1480,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1786095316</t>
+          <t>1786096483</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1490,7 +1490,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>15.69338</t>
+          <t>151.554007</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1507,12 +1507,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0xd6c7c9abba838597a4e77b3e2783253562734141d39ee275990cdeca84ed5917</t>
+          <t>0xfcb42550a86c19b2c5cb5270b8fbf7ab1826b37014cd165720a9eba42002beba</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0x8Aba6E6af9321Edf3b1b3b1CA92adEdb93D247C6</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1522,22 +1522,22 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>173</t>
+          <t>5.63</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.3438</t>
+          <t>1.3588</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Over 3.5</t>
+          <t>Excelsior Rotterdam FC</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1562,7 +1562,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0x5f73abff6c3a4dcbae7549384a24a6e32ed4fba83d1f8b6c07a54368215ec4b8</t>
+          <t>0xaa0c126d35fe767a756910f2acec4006318f8fe1dab75625727393f8adb31b74</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1592,7 +1592,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1786086947</t>
+          <t>1786095316</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1602,7 +1602,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>503.272727</t>
+          <t>15.69338</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1619,12 +1619,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x9f01fbafa94a70a9cf6ab60945073f6a9cfd9c030489c2f7ad0e408d82e12640</t>
+          <t>0xd6c7c9abba838597a4e77b3e2783253562734141d39ee275990cdeca84ed5917</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0xcF597434D48cDA55032b9d4931a0FFAeeEe7fb0D</t>
+          <t>0x8Aba6E6af9321Edf3b1b3b1CA92adEdb93D247C6</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1634,47 +1634,47 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>20.39624</t>
+          <t>173</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.375</t>
+          <t>1.3438</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (3.5)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
+          <t>Over 3.5</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Eredivisie</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Cambuur vs Excelsior Rotterdam FC</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Cambuur</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
           <t>Excelsior Rotterdam FC</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Eredivisie</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>Cambuur vs Excelsior Rotterdam FC</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>Cambuur</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>Excelsior Rotterdam FC</t>
-        </is>
-      </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0xaa0c126d35fe767a756910f2acec4006318f8fe1dab75625727393f8adb31b74</t>
+          <t>0x5f73abff6c3a4dcbae7549384a24a6e32ed4fba83d1f8b6c07a54368215ec4b8</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1704,7 +1704,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1786082661</t>
+          <t>1786086947</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1714,7 +1714,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>54.389973</t>
+          <t>503.272727</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1731,31 +1731,39 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x763d8974248de39c38179dce6fdf8aabf07c45a9532c44fd941f4ecaa4053020</t>
+          <t>0x9f01fbafa94a70a9cf6ab60945073f6a9cfd9c030489c2f7ad0e408d82e12640</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr"/>
+          <t>0xcF597434D48cDA55032b9d4931a0FFAeeEe7fb0D</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>14.19</t>
+          <t>20.39624</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.5675</t>
+          <t>1.375</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Asian Handicap (-2.5)</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Excelsior Rotterdam FC</t>
+        </is>
+      </c>
       <c r="H13" t="inlineStr">
         <is>
           <t>Eredivisie</t>
@@ -1763,27 +1771,27 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>PSV Eindhoven vs Fortuna Sittard</t>
+          <t>Cambuur vs Excelsior Rotterdam FC</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>PSV Eindhoven</t>
+          <t>Cambuur</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Fortuna Sittard</t>
+          <t>Excelsior Rotterdam FC</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0x793b0538f962d70a57b2c5c4acd58d7dd39a82bb4331ea1b3fa94033d70c07e7</t>
+          <t>0xaa0c126d35fe767a756910f2acec4006318f8fe1dab75625727393f8adb31b74</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>L19403946</t>
+          <t>L19403942</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1808,17 +1816,17 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1786076493</t>
+          <t>1786082661</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786125600</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>25.004405</t>
+          <t>54.389973</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1835,28 +1843,28 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0xbe3757de0d107fa27fec050f220d2720a303c2274c5053b041e64a8587c5429d</t>
+          <t>0x763d8974248de39c38179dce6fdf8aabf07c45a9532c44fd941f4ecaa4053020</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>42.19</t>
+          <t>14.19</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.6338</t>
+          <t>1.5675</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
+          <t>Asian Handicap (-2.5)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
@@ -1867,27 +1875,27 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Cambuur vs Excelsior Rotterdam FC</t>
+          <t>PSV Eindhoven vs Fortuna Sittard</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Cambuur</t>
+          <t>PSV Eindhoven</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Excelsior Rotterdam FC</t>
+          <t>Fortuna Sittard</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0x5f73abff6c3a4dcbae7549384a24a6e32ed4fba83d1f8b6c07a54368215ec4b8</t>
+          <t>0x793b0538f962d70a57b2c5c4acd58d7dd39a82bb4331ea1b3fa94033d70c07e7</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>L19403942</t>
+          <t>L19403946</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1912,17 +1920,17 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1786044588</t>
+          <t>1786076493</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>1786125600</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>66.571992</t>
+          <t>25.004405</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1939,110 +1947,214 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>0xbe3757de0d107fa27fec050f220d2720a303c2274c5053b041e64a8587c5429d</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>42.19</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>1.6338</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Eredivisie</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Cambuur vs Excelsior Rotterdam FC</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Cambuur</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Excelsior Rotterdam FC</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>0x5f73abff6c3a4dcbae7549384a24a6e32ed4fba83d1f8b6c07a54368215ec4b8</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>L19403942</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>1786044588</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>1786125600</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>66.571992</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>0x4ca810464ed1f6cc74ea5318f5d93dec93f4b441fa85a47c53e1f17f3dc3f2ff</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
         <is>
           <t>35.25</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>1.195</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>Tie</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="H16" t="inlineStr">
         <is>
           <t>Eredivisie</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t>NEC Nijmegen vs SC Telstar</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="J16" t="inlineStr">
         <is>
           <t>NEC Nijmegen</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t>SC Telstar</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="L16" t="inlineStr">
         <is>
           <t>0x32e22d2bad4d17213f93e2773019169fc54af66f0156ef2678851d836d908f54</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="M16" t="inlineStr">
         <is>
           <t>L19403940</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P15" t="inlineStr">
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R15" t="inlineStr">
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
         <is>
           <t>1786038454</t>
         </is>
       </c>
-      <c r="S15" t="inlineStr">
+      <c r="S16" t="inlineStr">
         <is>
           <t>1786199400</t>
         </is>
       </c>
-      <c r="T15" t="inlineStr">
+      <c r="T16" t="inlineStr">
         <is>
           <t>180.769231</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr">
+      <c r="U16" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V15" t="inlineStr">
+      <c r="V16" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-07 16:02:47 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Eredivisie/trades.xlsx
+++ b/data/sxbet/ligas/Eredivisie/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V16"/>
+  <dimension ref="A1:V25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,39 +531,31 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x30e80e0f179988de24d2dd1521c00c47b8a96c2e0b127f5b72b5656e3f3c392a</t>
+          <t>0xfaf4beff3b7f9403b40b5b13cdf01850a5090f98754d18ca5f83f066da413540</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0xFe080e9732dfD21D183C50e533A0B4b16021512a</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>19.97</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.5888</t>
+          <t>1.4563</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Go Ahead Eagles</t>
-        </is>
-      </c>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>Eredivisie</t>
@@ -571,27 +563,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Go Ahead Eagles vs Willem II Tilburg</t>
+          <t>Cambuur vs Excelsior Rotterdam FC</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Go Ahead Eagles</t>
+          <t>Cambuur</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Willem II Tilburg</t>
+          <t>Excelsior Rotterdam FC</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x8aa5f120fe51985c65586c394c669657f5118efb952dee047f9dabfcbeb011d3</t>
+          <t>0x16fabaade5687754bb46d8491b53388dc9815cef412e67a28d99cace1f9401a7</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19403947</t>
+          <t>L19403942</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -616,17 +608,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786111515</t>
+          <t>1786117951</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1786207500</t>
+          <t>1786125600</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1.698514</t>
+          <t>43.769863</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,39 +635,31 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x5814ac08c32ab173d1a31814cb3a6b884d7c9919e8f377ee4f05aeaa32cb47ee</t>
+          <t>0x5ded18ee9cf6d0038c25bfcf4cdaa513fe3f5574ccbf784436b2d6d1a93f94bb</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0xCf35f1782f282b1c6659882a3FAA48C637Ab693b</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xC3dd311005D417d573090717c8981A244b010aDc</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>9.99999</t>
+          <t>0.99998</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.5888</t>
+          <t>1.6812</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Go Ahead Eagles</t>
-        </is>
-      </c>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>Eredivisie</t>
@@ -683,27 +667,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Go Ahead Eagles vs Willem II Tilburg</t>
+          <t>Cambuur vs Excelsior Rotterdam FC</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Go Ahead Eagles</t>
+          <t>Cambuur</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Willem II Tilburg</t>
+          <t>Excelsior Rotterdam FC</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x8aa5f120fe51985c65586c394c669657f5118efb952dee047f9dabfcbeb011d3</t>
+          <t>0x5f73abff6c3a4dcbae7549384a24a6e32ed4fba83d1f8b6c07a54368215ec4b8</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19403947</t>
+          <t>L19403942</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -728,17 +712,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786105696</t>
+          <t>1786116835</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1786207500</t>
+          <t>1786125600</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>16.985121</t>
+          <t>1.467861</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -755,39 +739,31 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0xf98e5cfa7926a69ff6e557c416734c337a5cb9347da000cf0a1b8afd308312c1</t>
+          <t>0x4e752655ff6e177e1cb3bc0a594bc3d4797ae02f5942f50c529961f6934acd10</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0xCf35f1782f282b1c6659882a3FAA48C637Ab693b</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4.49993</t>
+          <t>3.45</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.9463</t>
+          <t>1.69</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Under/Over (0.5)</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Over 0.5</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>Eredivisie</t>
@@ -795,27 +771,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Cambuur vs Excelsior Rotterdam</t>
+          <t>FC Groningen vs FC Utrecht</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Cambuur</t>
+          <t>FC Groningen</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Excelsior Rotterdam</t>
+          <t>FC Utrecht</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x1decb278c23c8109eb9cf89c45fcff13cc3065960479465ded1dc8684e6e3f1f</t>
+          <t>0xade4255f0990d680e7f97af3f0657bc324f1ff60d7a5809184574fdacbbbb3be</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19403942</t>
+          <t>L19403944</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -840,17 +816,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786104752</t>
+          <t>1786115830</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1786125600</t>
+          <t>1786278600</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>4.75554</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -867,39 +843,31 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x85052153f0e8ac58dbcbeb02f546bbc166e1c5e3e8753d3dee4219a55150e22d</t>
+          <t>0xeda1b6d90374f6dfb1eb5db7e196f22b05428f1c82d7c343bc33c73b67266d78</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0xCf35f1782f282b1c6659882a3FAA48C637Ab693b</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.99989</t>
+          <t>1.36999</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.945</t>
+          <t>1.69</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Under/Over (0.5)</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Over 0.5</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>Eredivisie</t>
@@ -907,27 +875,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Cambuur vs Excelsior Rotterdam</t>
+          <t>FC Groningen vs FC Utrecht</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Cambuur</t>
+          <t>FC Groningen</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Excelsior Rotterdam</t>
+          <t>FC Utrecht</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0x1decb278c23c8109eb9cf89c45fcff13cc3065960479465ded1dc8684e6e3f1f</t>
+          <t>0xade4255f0990d680e7f97af3f0657bc324f1ff60d7a5809184574fdacbbbb3be</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19403942</t>
+          <t>L19403944</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -952,17 +920,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786104743</t>
+          <t>1786115829</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>1786125600</t>
+          <t>1786278600</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>6.34909</t>
+          <t>1.985493</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -979,28 +947,28 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0xc99b1deff403bd60532b3766c532f84759f6d39b1bdbf56a0da46442c81b8dbe</t>
+          <t>0x5a3f9702291c1ba964abe33fedccffcf9d3ad9537235ab7b839f5865be46b8a5</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0xbFA1723b261cB748697a7FFc3236E1c7C04bfC5e</t>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2.27</t>
+          <t>1.00999</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.6125</t>
+          <t>1.69</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Under/Over (4.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
@@ -1011,27 +979,27 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>PSV Eindhoven vs Fortuna Sittard</t>
+          <t>FC Groningen vs FC Utrecht</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>PSV Eindhoven</t>
+          <t>FC Groningen</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Fortuna Sittard</t>
+          <t>FC Utrecht</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0xd10635672e9e5618b0fee4290a52fdad51735dc4dfbd7ede4bc2a4e63cc90c47</t>
+          <t>0xade4255f0990d680e7f97af3f0657bc324f1ff60d7a5809184574fdacbbbb3be</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>L19403946</t>
+          <t>L19403944</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1056,17 +1024,17 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786102413</t>
+          <t>1786115827</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786278600</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>3.706122</t>
+          <t>1.463754</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1083,31 +1051,39 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x557b8c1f5c5c8b5fb903d079ecd882cabc34a595be512242ec8c9f410dc89cc8</t>
+          <t>0x766cd6df2eab89155d957f9e8c70e449311d87969614090438e8172ea68e472d</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0xbFA1723b261cB748697a7FFc3236E1c7C04bfC5e</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
+          <t>0x0DeAbC808957aBc9f4778C03b03CC1D2cBBC9D60</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.2212</t>
+          <t>1.3687</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Excelsior Rotterdam FC</t>
+        </is>
+      </c>
       <c r="H7" t="inlineStr">
         <is>
           <t>Eredivisie</t>
@@ -1115,27 +1091,27 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>PSV Eindhoven vs Fortuna Sittard</t>
+          <t>Cambuur vs Excelsior Rotterdam FC</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>PSV Eindhoven</t>
+          <t>Cambuur</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Fortuna Sittard</t>
+          <t>Excelsior Rotterdam FC</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x655963edf32f16b3a45d6a00e88736f6309fec1474356ce20fc40bcb6fec13aa</t>
+          <t>0xaa0c126d35fe767a756910f2acec4006318f8fe1dab75625727393f8adb31b74</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>L19403946</t>
+          <t>L19403942</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1160,17 +1136,17 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786102412</t>
+          <t>1786115129</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786125600</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>4.519774</t>
+          <t>13.559322</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1187,28 +1163,28 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0xd876072232054549cb6720da6ed0929158b37dc7f9e1ed70e03cf4bb6785214e</t>
+          <t>0x1c3956d4fd671eb8f64e9c1dde1907d26d4ca3284611bf2166ba25878ada840d</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0xbFA1723b261cB748697a7FFc3236E1c7C04bfC5e</t>
+          <t>0x0DeAbC808957aBc9f4778C03b03CC1D2cBBC9D60</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.4138</t>
+          <t>1.5075</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
+          <t>Eredivisie</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
@@ -1219,27 +1195,27 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>PSV Eindhoven vs Fortuna Sittard</t>
+          <t>Cambuur vs Excelsior Rotterdam FC</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>PSV Eindhoven</t>
+          <t>Cambuur</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Fortuna Sittard</t>
+          <t>Excelsior Rotterdam FC</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x8e63f170dc54d5f8c63f531a5dcccded818e9d9e5f10a9596397c42875b381c7</t>
+          <t>0x9ab95655b7491fc8e615c8d50d6b5fe19a0750663b098d28624ff47a889afa65</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>L19403946</t>
+          <t>L19403942</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1264,17 +1240,17 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1786102410</t>
+          <t>1786115128</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786125600</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>2.416918</t>
+          <t>9.852217</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1291,31 +1267,39 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0xfb67071ab7e9a27f540fd95f339b51a0fac006bd9950b6d733ec4be68c85bb16</t>
+          <t>0xd45d17af5b95ec1c1350bb1787486845b1e75220b35567f190918eb7f442b573</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0xbFA1723b261cB748697a7FFc3236E1c7C04bfC5e</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>31.38</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.195</t>
+          <t>1.3675</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Excelsior Rotterdam FC</t>
+        </is>
+      </c>
       <c r="H9" t="inlineStr">
         <is>
           <t>Eredivisie</t>
@@ -1323,27 +1307,27 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Go Ahead Eagles vs Willem II Tilburg</t>
+          <t>Cambuur vs Excelsior Rotterdam FC</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Go Ahead Eagles</t>
+          <t>Cambuur</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Willem II Tilburg</t>
+          <t>Excelsior Rotterdam FC</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0x850e00f49e80137284f56035827d7137ff8b0500f064e9bbebfb9172d34d807c</t>
+          <t>0xaa0c126d35fe767a756910f2acec4006318f8fe1dab75625727393f8adb31b74</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>L19403947</t>
+          <t>L19403942</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1368,17 +1352,17 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1786102409</t>
+          <t>1786115115</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>1786207500</t>
+          <t>1786125600</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>5.128205</t>
+          <t>85.387755</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1395,62 +1379,54 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0xe3ab30d6b781a9a79b98b5a3c156060adf02a4cb6dd79257d045954564c464f4</t>
+          <t>0xc314db881b3e02a32691c317283fd9a8fdab70d92c17be01a655abfdbd237005</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>54.37</t>
+          <t>177.44126</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.3588</t>
+          <t>1.5063</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
+          <t>Eredivisie</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Eredivisie</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Cambuur vs Excelsior Rotterdam FC</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Cambuur</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
         <is>
           <t>Excelsior Rotterdam FC</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Eredivisie</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>Cambuur vs Excelsior Rotterdam FC</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>Cambuur</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>Excelsior Rotterdam FC</t>
-        </is>
-      </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0xaa0c126d35fe767a756910f2acec4006318f8fe1dab75625727393f8adb31b74</t>
+          <t>0x9ab95655b7491fc8e615c8d50d6b5fe19a0750663b098d28624ff47a889afa65</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1480,7 +1456,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1786096483</t>
+          <t>1786115115</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1490,7 +1466,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>151.554007</t>
+          <t>350.501254</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1507,12 +1483,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0xfcb42550a86c19b2c5cb5270b8fbf7ab1826b37014cd165720a9eba42002beba</t>
+          <t>0x30e80e0f179988de24d2dd1521c00c47b8a96c2e0b127f5b72b5656e3f3c392a</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0xFe080e9732dfD21D183C50e533A0B4b16021512a</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1522,12 +1498,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>5.63</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.3588</t>
+          <t>1.5888</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1537,7 +1513,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Excelsior Rotterdam FC</t>
+          <t>Go Ahead Eagles</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1547,27 +1523,27 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Cambuur vs Excelsior Rotterdam FC</t>
+          <t>Go Ahead Eagles vs Willem II Tilburg</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Cambuur</t>
+          <t>Go Ahead Eagles</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Excelsior Rotterdam FC</t>
+          <t>Willem II Tilburg</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0xaa0c126d35fe767a756910f2acec4006318f8fe1dab75625727393f8adb31b74</t>
+          <t>0x8aa5f120fe51985c65586c394c669657f5118efb952dee047f9dabfcbeb011d3</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>L19403942</t>
+          <t>L19403947</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1592,17 +1568,17 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1786095316</t>
+          <t>1786111515</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>1786125600</t>
+          <t>1786207500</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>15.69338</t>
+          <t>1.698514</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1619,12 +1595,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0xd6c7c9abba838597a4e77b3e2783253562734141d39ee275990cdeca84ed5917</t>
+          <t>0x5814ac08c32ab173d1a31814cb3a6b884d7c9919e8f377ee4f05aeaa32cb47ee</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0x8Aba6E6af9321Edf3b1b3b1CA92adEdb93D247C6</t>
+          <t>0xCf35f1782f282b1c6659882a3FAA48C637Ab693b</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1634,22 +1610,22 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>173</t>
+          <t>9.99999</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.3438</t>
+          <t>1.5888</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Over 3.5</t>
+          <t>Go Ahead Eagles</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1659,27 +1635,27 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Cambuur vs Excelsior Rotterdam FC</t>
+          <t>Go Ahead Eagles vs Willem II Tilburg</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Cambuur</t>
+          <t>Go Ahead Eagles</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Excelsior Rotterdam FC</t>
+          <t>Willem II Tilburg</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0x5f73abff6c3a4dcbae7549384a24a6e32ed4fba83d1f8b6c07a54368215ec4b8</t>
+          <t>0x8aa5f120fe51985c65586c394c669657f5118efb952dee047f9dabfcbeb011d3</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>L19403942</t>
+          <t>L19403947</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1704,17 +1680,17 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1786086947</t>
+          <t>1786105696</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>1786125600</t>
+          <t>1786207500</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>503.272727</t>
+          <t>16.985121</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1731,12 +1707,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x9f01fbafa94a70a9cf6ab60945073f6a9cfd9c030489c2f7ad0e408d82e12640</t>
+          <t>0xf98e5cfa7926a69ff6e557c416734c337a5cb9347da000cf0a1b8afd308312c1</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0xcF597434D48cDA55032b9d4931a0FFAeeEe7fb0D</t>
+          <t>0xCf35f1782f282b1c6659882a3FAA48C637Ab693b</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1746,22 +1722,22 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>20.39624</t>
+          <t>4.49993</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.375</t>
+          <t>1.9463</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (0.5)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Excelsior Rotterdam FC</t>
+          <t>Over 0.5</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1771,7 +1747,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Cambuur vs Excelsior Rotterdam FC</t>
+          <t>Cambuur vs Excelsior Rotterdam</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1781,12 +1757,12 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Excelsior Rotterdam FC</t>
+          <t>Excelsior Rotterdam</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0xaa0c126d35fe767a756910f2acec4006318f8fe1dab75625727393f8adb31b74</t>
+          <t>0x1decb278c23c8109eb9cf89c45fcff13cc3065960479465ded1dc8684e6e3f1f</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1816,7 +1792,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1786082661</t>
+          <t>1786104752</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1826,7 +1802,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>54.389973</t>
+          <t>4.75554</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1843,31 +1819,39 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0x763d8974248de39c38179dce6fdf8aabf07c45a9532c44fd941f4ecaa4053020</t>
+          <t>0x85052153f0e8ac58dbcbeb02f546bbc166e1c5e3e8753d3dee4219a55150e22d</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr"/>
+          <t>0xCf35f1782f282b1c6659882a3FAA48C637Ab693b</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>14.19</t>
+          <t>5.99989</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.5675</t>
+          <t>1.945</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Asian Handicap (-2.5)</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr"/>
+          <t>Under/Over (0.5)</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Over 0.5</t>
+        </is>
+      </c>
       <c r="H14" t="inlineStr">
         <is>
           <t>Eredivisie</t>
@@ -1875,27 +1859,27 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>PSV Eindhoven vs Fortuna Sittard</t>
+          <t>Cambuur vs Excelsior Rotterdam</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>PSV Eindhoven</t>
+          <t>Cambuur</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Fortuna Sittard</t>
+          <t>Excelsior Rotterdam</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0x793b0538f962d70a57b2c5c4acd58d7dd39a82bb4331ea1b3fa94033d70c07e7</t>
+          <t>0x1decb278c23c8109eb9cf89c45fcff13cc3065960479465ded1dc8684e6e3f1f</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>L19403946</t>
+          <t>L19403942</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1920,17 +1904,17 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1786076493</t>
+          <t>1786104743</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786125600</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>25.004405</t>
+          <t>6.34909</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1947,28 +1931,28 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0xbe3757de0d107fa27fec050f220d2720a303c2274c5053b041e64a8587c5429d</t>
+          <t>0xc99b1deff403bd60532b3766c532f84759f6d39b1bdbf56a0da46442c81b8dbe</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0xbFA1723b261cB748697a7FFc3236E1c7C04bfC5e</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>42.19</t>
+          <t>2.27</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.6338</t>
+          <t>1.6125</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
+          <t>Under/Over (4.5)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
@@ -1979,27 +1963,27 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Cambuur vs Excelsior Rotterdam FC</t>
+          <t>PSV Eindhoven vs Fortuna Sittard</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Cambuur</t>
+          <t>PSV Eindhoven</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Excelsior Rotterdam FC</t>
+          <t>Fortuna Sittard</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0x5f73abff6c3a4dcbae7549384a24a6e32ed4fba83d1f8b6c07a54368215ec4b8</t>
+          <t>0xd10635672e9e5618b0fee4290a52fdad51735dc4dfbd7ede4bc2a4e63cc90c47</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>L19403942</t>
+          <t>L19403946</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -2024,17 +2008,17 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1786044588</t>
+          <t>1786102413</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>1786125600</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>66.571992</t>
+          <t>3.706122</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2051,110 +2035,1078 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>0x557b8c1f5c5c8b5fb903d079ecd882cabc34a595be512242ec8c9f410dc89cc8</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>0xbFA1723b261cB748697a7FFc3236E1c7C04bfC5e</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>1.2212</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Eredivisie</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>PSV Eindhoven vs Fortuna Sittard</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>PSV Eindhoven</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Fortuna Sittard</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>0x655963edf32f16b3a45d6a00e88736f6309fec1474356ce20fc40bcb6fec13aa</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>L19403946</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>1786102412</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>1786212000</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>4.519774</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>0xd876072232054549cb6720da6ed0929158b37dc7f9e1ed70e03cf4bb6785214e</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>0xbFA1723b261cB748697a7FFc3236E1c7C04bfC5e</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>1.4138</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Eredivisie</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>PSV Eindhoven vs Fortuna Sittard</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>PSV Eindhoven</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Fortuna Sittard</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>0x8e63f170dc54d5f8c63f531a5dcccded818e9d9e5f10a9596397c42875b381c7</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>L19403946</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>1786102410</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>1786212000</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>2.416918</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>0xfb67071ab7e9a27f540fd95f339b51a0fac006bd9950b6d733ec4be68c85bb16</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>0xbFA1723b261cB748697a7FFc3236E1c7C04bfC5e</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>1.195</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Eredivisie</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Go Ahead Eagles vs Willem II Tilburg</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Go Ahead Eagles</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Willem II Tilburg</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>0x850e00f49e80137284f56035827d7137ff8b0500f064e9bbebfb9172d34d807c</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>L19403947</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>1786102409</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>1786207500</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>5.128205</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>0xe3ab30d6b781a9a79b98b5a3c156060adf02a4cb6dd79257d045954564c464f4</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>54.37</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>1.3588</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Excelsior Rotterdam FC</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Eredivisie</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Cambuur vs Excelsior Rotterdam FC</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Cambuur</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Excelsior Rotterdam FC</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>0xaa0c126d35fe767a756910f2acec4006318f8fe1dab75625727393f8adb31b74</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>L19403942</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>1786096483</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>1786125600</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>151.554007</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>0xfcb42550a86c19b2c5cb5270b8fbf7ab1826b37014cd165720a9eba42002beba</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>5.63</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>1.3588</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Excelsior Rotterdam FC</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Eredivisie</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Cambuur vs Excelsior Rotterdam FC</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Cambuur</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Excelsior Rotterdam FC</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>0xaa0c126d35fe767a756910f2acec4006318f8fe1dab75625727393f8adb31b74</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>L19403942</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>1786095316</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>1786125600</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>15.69338</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>0xd6c7c9abba838597a4e77b3e2783253562734141d39ee275990cdeca84ed5917</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>0x8Aba6E6af9321Edf3b1b3b1CA92adEdb93D247C6</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>173</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>1.3438</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Over 3.5</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Eredivisie</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Cambuur vs Excelsior Rotterdam FC</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Cambuur</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Excelsior Rotterdam FC</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>0x5f73abff6c3a4dcbae7549384a24a6e32ed4fba83d1f8b6c07a54368215ec4b8</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>L19403942</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>1786086947</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>1786125600</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>503.272727</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>0x9f01fbafa94a70a9cf6ab60945073f6a9cfd9c030489c2f7ad0e408d82e12640</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>0xcF597434D48cDA55032b9d4931a0FFAeeEe7fb0D</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>20.39624</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>1.375</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Excelsior Rotterdam FC</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Eredivisie</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Cambuur vs Excelsior Rotterdam FC</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Cambuur</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Excelsior Rotterdam FC</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>0xaa0c126d35fe767a756910f2acec4006318f8fe1dab75625727393f8adb31b74</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>L19403942</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>1786082661</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>1786125600</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>54.389973</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>0x763d8974248de39c38179dce6fdf8aabf07c45a9532c44fd941f4ecaa4053020</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>14.19</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>1.5675</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-2.5)</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Eredivisie</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>PSV Eindhoven vs Fortuna Sittard</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>PSV Eindhoven</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Fortuna Sittard</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>0x793b0538f962d70a57b2c5c4acd58d7dd39a82bb4331ea1b3fa94033d70c07e7</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>L19403946</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>1786076493</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>1786212000</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>25.004405</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>0xbe3757de0d107fa27fec050f220d2720a303c2274c5053b041e64a8587c5429d</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>42.19</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>1.6338</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Eredivisie</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Cambuur vs Excelsior Rotterdam FC</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Cambuur</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Excelsior Rotterdam FC</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>0x5f73abff6c3a4dcbae7549384a24a6e32ed4fba83d1f8b6c07a54368215ec4b8</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>L19403942</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>1786044588</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>1786125600</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>66.571992</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>0x4ca810464ed1f6cc74ea5318f5d93dec93f4b441fa85a47c53e1f17f3dc3f2ff</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
         <is>
           <t>35.25</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>1.195</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F25" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="G25" t="inlineStr">
         <is>
           <t>Tie</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="H25" t="inlineStr">
         <is>
           <t>Eredivisie</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="I25" t="inlineStr">
         <is>
           <t>NEC Nijmegen vs SC Telstar</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="J25" t="inlineStr">
         <is>
           <t>NEC Nijmegen</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="K25" t="inlineStr">
         <is>
           <t>SC Telstar</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
+      <c r="L25" t="inlineStr">
         <is>
           <t>0x32e22d2bad4d17213f93e2773019169fc54af66f0156ef2678851d836d908f54</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
+      <c r="M25" t="inlineStr">
         <is>
           <t>L19403940</t>
         </is>
       </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P16" t="inlineStr">
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R16" t="inlineStr">
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
         <is>
           <t>1786038454</t>
         </is>
       </c>
-      <c r="S16" t="inlineStr">
+      <c r="S25" t="inlineStr">
         <is>
           <t>1786199400</t>
         </is>
       </c>
-      <c r="T16" t="inlineStr">
+      <c r="T25" t="inlineStr">
         <is>
           <t>180.769231</t>
         </is>
       </c>
-      <c r="U16" t="inlineStr">
+      <c r="U25" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V16" t="inlineStr">
+      <c r="V25" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>